<commit_message>
Implement comprehensive restriction rules management including frontend components, services, and backend integration.
</commit_message>
<xml_diff>
--- a/import-examples/timetable_data.xlsx
+++ b/import-examples/timetable_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diallofrancispatrick/Desktop/workspace/Automatic-Timetable-Generation-System/import-examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81886E9B-10E5-0C4D-AFAF-2FB8F89CAF08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD0F70D3-FE7A-6349-975F-0321330DAA8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16180" activeTab="4" xr2:uid="{463DB273-5E57-1240-BC5F-E8CC45185236}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16140" activeTab="4" xr2:uid="{463DB273-5E57-1240-BC5F-E8CC45185236}"/>
   </bookViews>
   <sheets>
     <sheet name="Timeslots" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="StudentGroups" sheetId="4" r:id="rId4"/>
     <sheet name="Lessons" sheetId="5" r:id="rId5"/>
     <sheet name="Configuration" sheetId="6" r:id="rId6"/>
+    <sheet name="RestrictionRules" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="58">
   <si>
     <t>id</t>
   </si>
@@ -173,6 +174,48 @@
   </si>
   <si>
     <t>roomId</t>
+  </si>
+  <si>
+    <t>targetType</t>
+  </si>
+  <si>
+    <t>criteriaField</t>
+  </si>
+  <si>
+    <t>operator</t>
+  </si>
+  <si>
+    <t>criteriaValue</t>
+  </si>
+  <si>
+    <t>active</t>
+  </si>
+  <si>
+    <t>Morning Only</t>
+  </si>
+  <si>
+    <t>TIMESLOT</t>
+  </si>
+  <si>
+    <t>START_TIME</t>
+  </si>
+  <si>
+    <t>LESS_THAN</t>
+  </si>
+  <si>
+    <t>Big Rooms</t>
+  </si>
+  <si>
+    <t>ROOM</t>
+  </si>
+  <si>
+    <t>CAPACITY</t>
+  </si>
+  <si>
+    <t>GREATER_THAN</t>
+  </si>
+  <si>
+    <t>appliedRuleIds</t>
   </si>
 </sst>
 </file>
@@ -219,7 +262,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -227,6 +270,7 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -816,16 +860,17 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CBC01F1-606B-AC4B-9826-7C03E429838C}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="14.5" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
     <col min="7" max="7" width="13.6640625" customWidth="1"/>
+    <col min="11" max="11" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -856,8 +901,11 @@
       <c r="J1" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K1" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -882,8 +930,11 @@
       <c r="H2" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K2">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -909,7 +960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -935,7 +986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>6</v>
       </c>
@@ -1024,4 +1075,89 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9F5C8B9-A3F5-0C42-B782-A97265210A08}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>102</v>
+      </c>
+      <c r="B3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3">
+        <v>100</v>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
 </file>
</xml_diff>